<commit_message>
Order update: Nolan Crockford bought + paid for #008, #015, #030, #035, #097
</commit_message>
<xml_diff>
--- a/disc-pics-data/Disc Diver Sales Tracker.xlsx
+++ b/disc-pics-data/Disc Diver Sales Tracker.xlsx
@@ -511,7 +511,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>12 sold  •  $112 total  •  $0 collected  •  12 still to ship</t>
+          <t>12 sold  •  $112 total  •  $43 collected  •  12 still to ship</t>
         </is>
       </c>
     </row>
@@ -639,10 +639,14 @@
       <c r="E6" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="F6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Nolan Crockford</t>
+        </is>
+      </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -764,10 +768,14 @@
       <c r="E9" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="F9" s="5" t="inlineStr"/>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Nolan Crockford</t>
+        </is>
+      </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -807,10 +815,14 @@
       <c r="E10" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="F10" s="5" t="inlineStr"/>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Nolan Crockford</t>
+        </is>
+      </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -846,10 +858,14 @@
       <c r="E11" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="F11" s="5" t="inlineStr"/>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Nolan Crockford</t>
+        </is>
+      </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1069,10 +1085,14 @@
       <c r="E16" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="F16" s="5" t="inlineStr"/>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Nolan Crockford</t>
+        </is>
+      </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Note S&H paid on Nolan Crockford's combined order
</commit_message>
<xml_diff>
--- a/disc-pics-data/Disc Diver Sales Tracker.xlsx
+++ b/disc-pics-data/Disc Diver Sales Tracker.xlsx
@@ -660,7 +660,11 @@
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr"/>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>paid $43 + S&amp;H (combined ship)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -789,7 +793,11 @@
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr"/>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>paid $43 + S&amp;H (combined ship)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -836,7 +844,11 @@
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="K10" s="5" t="inlineStr"/>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>paid $43 + S&amp;H (combined ship)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -879,7 +891,11 @@
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="K11" s="5" t="inlineStr"/>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>paid $43 + S&amp;H (combined ship)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1106,7 +1122,11 @@
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="K16" s="5" t="inlineStr"/>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>paid $43 + S&amp;H (combined ship)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="G5:G16">

</xml_diff>